<commit_message>
Fill HSK2 parts 4 (ID 651-700) with parts of speech
</commit_message>
<xml_diff>
--- a/HSK2_parts_of_speech_4(651-700).xlsx
+++ b/HSK2_parts_of_speech_4(651-700).xlsx
@@ -644,6 +644,21 @@
           <t>большинство</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>большинство</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>многочисленный (多数的例子 — 多数例子)</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>от 多; антоним 少数</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -670,6 +685,16 @@
           <t>облачно</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>пасмурная погода</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>облачно (небо)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -696,6 +721,16 @@
           <t>к тому же</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>а к тому же, притом</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>усилительный союз во второй части (不但…而且…)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -722,6 +757,21 @@
           <t>отправлять, выпускать</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>отправлять; выпускать;发出(издавать звук); 发烧(температу­рить), 发明(изобретать)</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>для выстрелов/вспышек (打了一发子弹)</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>离合词 основа: 发财, 生病等 сочетания; само разъединяется: 发了一次言</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -748,6 +798,11 @@
           <t>обнаруживать</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>обнаруживать, находить</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -774,6 +829,11 @@
           <t>кафе, ресторан</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ресторан, кафе (небольшой)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -800,6 +860,21 @@
           <t>удобный</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>быть удобным (方便一下 — отлучиться)</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>удобный; сподручный</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>при вежливом отказе 不太方便 = «неудобно»</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -826,6 +901,11 @@
           <t>лапша быстрого приготовления</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>лапша быстрого приготовления</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -852,6 +932,16 @@
           <t>метод, приём</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>метод, способ</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>для методов (一种方法)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -878,6 +968,21 @@
           <t>сторона, аспект</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>сторона, аспект</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>в области…, по части… (动力方面 — в отношении движущей силы)</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>после слова образует «по такой-то стороне»</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -904,6 +1009,11 @@
           <t>направление</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>направление</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -930,6 +1040,16 @@
           <t>отпустить, положить</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>положить (вниз),放下; отпустить</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>глагол + результативное дополнение 下; разъединяется: 把书放下来</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -956,6 +1076,16 @@
           <t>быть спокойным</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>быть спокойным, не беспокоиться</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>离合词 (动宾): 放心吧, 别放心不下</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -982,6 +1112,26 @@
           <t>делить</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>минута (время); очко, балл</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>делить; разделения</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>для денег: фэнь = 0,01 юаня</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>многозначное: fēn — делить, fèn — доля/成分; 一分钟, 三分之…</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1008,6 +1158,16 @@
           <t>разделять, отрывать</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>разделять, разлучить</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>глагол + результативное дополнение 开: 分开了三年</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1034,6 +1194,11 @@
           <t>балл, отметка; дробь</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>оценка, балл; дробь</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1060,6 +1225,11 @@
           <t>минута</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>минута (единица времени)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1086,6 +1256,16 @@
           <t>часть, доля</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>часть, доля (股份)</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>доля, экземпляр (一份报纸, 两份合同)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1112,6 +1292,26 @@
           <t>счётное слово для писем</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>конверт; печать (封住)</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>запечатывать</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>для писем (一封信)</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>как 名/гл — книжное/устаревшее (封疆); частотное — счётное слово</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1138,6 +1338,21 @@
           <t>обслуживать; услуга</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>сервис, обслуживание</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>обслуживать</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>служебный (服务员 — официант)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1164,6 +1379,11 @@
           <t>повторять, упражняться</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>повторять (пройденное), повторяться</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1190,6 +1410,21 @@
           <t>быть должным, следует</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>должный, следует (应该)</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>как раз тот (该人 — данный)</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>обычно в связке 应该; одиночное 该 книжное</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1216,6 +1451,11 @@
           <t>изменять, исправлять</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>исправлять, изменять (改错, 改名)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1242,6 +1482,16 @@
           <t>изменять, преобразовывать</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>изменять, преобразовывать</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>ближе к «трансформировать», чем бытовое 改</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1268,6 +1518,16 @@
           <t>выпить до дна</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>чокнуться, выпить до дна (тост)</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>离合词 (动宾): 干一杯!</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1294,6 +1554,16 @@
           <t>почувствовать</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>чувствовать, ощущать (感到高兴)</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>грамматическая конструкция: 感+到 — глагол с результатом; синонимично 觉得</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1320,6 +1590,16 @@
           <t>растрогать, воодушевить</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>растрогать, тронуть (被感动)</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>трогательный (很感动)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1346,6 +1626,16 @@
           <t>чувство; чувствовать</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>чувство, ощущение</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>чувствовать, ощущать</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1372,6 +1662,21 @@
           <t>благодарить</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>благодарность</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>благодарить (表示感谢)</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>более формальное, чем 谢谢</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1398,6 +1703,16 @@
           <t>работать, трудиться</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>работать, трудиться (физически)</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>离合词 (动宾) с erhua: 干了一天活儿</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1424,6 +1739,21 @@
           <t>твёрдый; только что</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>твердый (刚的馒头)</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>только что (刚来)</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>жесткий, прямой (刚直)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1450,6 +1780,21 @@
           <t>только что</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>момент только что (时间词)</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>только что</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>только о прошедшем; нельзя *刚才没来</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1476,6 +1821,16 @@
           <t>только что, едва-едва</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>самый свежий/ровный (刚刚的事)</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>только что, едва</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1502,6 +1857,16 @@
           <t>высокий уровень</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>высокого уровня, премиум (高级酒店)</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>старший/высший (高级工程师)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1528,6 +1893,11 @@
           <t>высшая ступень средней школы</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>последние классы средней школы (10–12)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1554,6 +1924,16 @@
           <t>рост</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>рост (человека)</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>в паре 个子: 他个子很高; 个 здесь — безударный аффикс</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1580,6 +1960,21 @@
           <t>более</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>другой? нет — см. 更(gēng) «менять» редк.</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>ещё более, гораздо (更好)</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>gèng — только наречие «ещё более»; книж. gēng «менять» (更替) в HSK не входит</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1606,6 +2001,11 @@
           <t>автобус</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>автобус</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1632,6 +2032,11 @@
           <t>общественный транспорт</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>городской автобус/общественный транспорт</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1658,6 +2063,11 @@
           <t>килограмм</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>килограмм</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1684,6 +2094,11 @@
           <t>километр</t>
         </is>
       </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>километр</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1710,6 +2125,11 @@
           <t>шоссе</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>шоссе, автодорога</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1736,6 +2156,16 @@
           <t>справедливый</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>справедливость (讲公平)</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>справедливый, беспристрастный</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1762,6 +2192,11 @@
           <t>компания</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>компания, фирма</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1788,6 +2223,11 @@
           <t>парк</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>парк</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1814,6 +2254,11 @@
           <t>собака</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>собака</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1840,6 +2285,21 @@
           <t>достаточно</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>достигать (够得着 — дотянуться)</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>достаточно (人够了)</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>вполне, достаточно (够意思 — ты молодец)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1866,6 +2326,11 @@
           <t>история, рассказ</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>история, рассказ, сюжет</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1892,6 +2357,21 @@
           <t>намеренно</t>
         </is>
       </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>преднамеренный (故意的行为)</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>намеренно, нарочно</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>сущ. 故意 (юр.) «умысел» — книжное</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1916,6 +2396,16 @@
       <c r="I51" t="inlineStr">
         <is>
           <t>клиент, покупатель</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>клиент, покупатель</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>служебное слово продавца</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix stray cell in HSK2 parts 4 (ID 687)
</commit_message>
<xml_diff>
--- a/HSK2_parts_of_speech_4(651-700).xlsx
+++ b/HSK2_parts_of_speech_4(651-700).xlsx
@@ -1960,11 +1960,6 @@
           <t>более</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>другой? нет — см. 更(gēng) «менять» редк.</t>
-        </is>
-      </c>
       <c r="Q38" t="inlineStr">
         <is>
           <t>ещё более, гораздо (更好)</t>

</xml_diff>